<commit_message>
Commit-3-SA Questions Evaluation Added
</commit_message>
<xml_diff>
--- a/answer.xlsx
+++ b/answer.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="25">
   <si>
     <t xml:space="preserve">Question id</t>
   </si>
@@ -68,6 +68,33 @@
   </si>
   <si>
     <t xml:space="preserve">SA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Naecoocean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">polarpolar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ghjemakbclifd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[(1,2),(2,1),(2,4),(3,0),(3,3),(4,2),(5,1),(5,4)]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[6,3,4,8,2,9]</t>
   </si>
 </sst>
 </file>
@@ -143,10 +170,18 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -343,650 +378,677 @@
   <dimension ref="A1:E41"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.82"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>6406531910667</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E2" s="0" t="s">
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>6406531910668</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E3" s="0" t="s">
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>6406531910669</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E4" s="0" t="s">
+      <c r="C4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>6406531910670</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E5" s="0" t="s">
+      <c r="C5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>6406531910671</v>
       </c>
-      <c r="B6" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E6" s="0" t="s">
+      <c r="B6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6406531910672</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C7" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E7" s="0" t="s">
+      <c r="C7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>6406531910673</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C8" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E8" s="0" t="s">
+      <c r="C8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>6406531910674</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C9" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E9" s="0" t="s">
+      <c r="C9" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
+      <c r="A10" s="1" t="n">
         <v>6406531910675</v>
       </c>
-      <c r="B10" s="0" t="n">
+      <c r="B10" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="C10" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D10" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E10" s="0" t="s">
+      <c r="C10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
+      <c r="A11" s="1" t="n">
         <v>6406531910676</v>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="C11" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E11" s="0" t="s">
+      <c r="C11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="n">
+      <c r="A12" s="1" t="n">
         <v>6406531910677</v>
       </c>
-      <c r="B12" s="0" t="n">
+      <c r="B12" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="C12" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E12" s="0" t="s">
+      <c r="C12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="n">
+      <c r="A13" s="1" t="n">
         <v>6406531910678</v>
       </c>
-      <c r="B13" s="0" t="n">
+      <c r="B13" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="C13" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D13" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E13" s="0" t="s">
+      <c r="C13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="n">
+      <c r="A14" s="1" t="n">
         <v>6406531910679</v>
       </c>
-      <c r="B14" s="0" t="n">
+      <c r="B14" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="C14" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D14" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E14" s="0" t="s">
+      <c r="C14" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="n">
+      <c r="A15" s="1" t="n">
         <v>6406531910680</v>
       </c>
-      <c r="B15" s="0" t="n">
+      <c r="B15" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="C15" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D15" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E15" s="0" t="s">
+      <c r="C15" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="n">
+      <c r="A16" s="1" t="n">
         <v>6406531910681</v>
       </c>
-      <c r="B16" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="C16" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D16" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E16" s="0" t="s">
+      <c r="B16" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="n">
+      <c r="A17" s="1" t="n">
         <v>6406531910683</v>
       </c>
-      <c r="B17" s="0" t="n">
+      <c r="B17" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="C17" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D17" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E17" s="0" t="s">
+      <c r="C17" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="n">
+      <c r="A18" s="1" t="n">
         <v>6406531910684</v>
       </c>
-      <c r="B18" s="0" t="n">
+      <c r="B18" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="C18" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E18" s="0" t="s">
+      <c r="C18" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="n">
+      <c r="A19" s="1" t="n">
         <v>6406531910686</v>
       </c>
-      <c r="B19" s="0" t="n">
+      <c r="B19" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="C19" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D19" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E19" s="0" t="s">
+      <c r="C19" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="n">
+      <c r="A20" s="1" t="n">
         <v>6406531910687</v>
       </c>
-      <c r="B20" s="0" t="n">
+      <c r="B20" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="C20" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D20" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E20" s="0" t="s">
+      <c r="C20" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D20" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="n">
+      <c r="A21" s="1" t="n">
         <v>6406531910689</v>
       </c>
-      <c r="B21" s="0" t="n">
+      <c r="B21" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="C21" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D21" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E21" s="0" t="s">
+      <c r="C21" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="n">
+      <c r="A22" s="1" t="n">
         <v>6406531910690</v>
       </c>
-      <c r="B22" s="0" t="n">
+      <c r="B22" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="C22" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E22" s="0" t="s">
+      <c r="C22" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="n">
+      <c r="A23" s="1" t="n">
         <v>6406531910691</v>
       </c>
-      <c r="B23" s="0" t="n">
+      <c r="B23" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="C23" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D23" s="0" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E23" s="0" t="s">
+      <c r="C23" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="n">
+      <c r="A24" s="1" t="n">
         <v>6406531910692</v>
       </c>
-      <c r="B24" s="0" t="n">
+      <c r="B24" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="C24" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D24" s="0" t="n">
-        <v>2.5</v>
+      <c r="C24" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="n">
+      <c r="A25" s="1" t="n">
         <v>6406531910693</v>
       </c>
-      <c r="B25" s="0" t="n">
+      <c r="B25" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="C25" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D25" s="0" t="n">
-        <v>2.5</v>
+      <c r="C25" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="n">
+      <c r="A26" s="1" t="n">
         <v>6406531910694</v>
       </c>
-      <c r="B26" s="0" t="n">
+      <c r="B26" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="C26" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D26" s="0" t="n">
-        <v>2.5</v>
+      <c r="C26" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="n">
+      <c r="A27" s="1" t="n">
         <v>6406531910695</v>
       </c>
-      <c r="B27" s="0" t="n">
+      <c r="B27" s="1" t="n">
         <v>26</v>
       </c>
-      <c r="C27" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D27" s="0" t="n">
-        <v>2.5</v>
+      <c r="C27" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="n">
+      <c r="A28" s="1" t="n">
         <v>6406531910696</v>
       </c>
-      <c r="B28" s="0" t="n">
+      <c r="B28" s="1" t="n">
         <v>27</v>
       </c>
-      <c r="C28" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D28" s="0" t="n">
-        <v>2.5</v>
+      <c r="C28" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="n">
+      <c r="A29" s="1" t="n">
         <v>6406531910697</v>
       </c>
-      <c r="B29" s="0" t="n">
+      <c r="B29" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="C29" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D29" s="0" t="n">
-        <v>2.5</v>
+      <c r="C29" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="n">
+      <c r="A30" s="1" t="n">
         <v>6406531910698</v>
       </c>
-      <c r="B30" s="0" t="n">
+      <c r="B30" s="1" t="n">
         <v>29</v>
       </c>
-      <c r="C30" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D30" s="0" t="n">
-        <v>2.5</v>
+      <c r="C30" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="n">
+      <c r="A31" s="1" t="n">
         <v>6406531910699</v>
       </c>
-      <c r="B31" s="0" t="n">
+      <c r="B31" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="C31" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D31" s="0" t="n">
-        <v>2.5</v>
+      <c r="C31" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="n">
+      <c r="A32" s="1" t="n">
         <v>6406531910700</v>
       </c>
-      <c r="B32" s="0" t="n">
+      <c r="B32" s="1" t="n">
         <v>31</v>
       </c>
-      <c r="C32" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D32" s="0" t="n">
-        <v>2.5</v>
+      <c r="C32" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D32" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="n">
+      <c r="A33" s="1" t="n">
         <v>6406531910702</v>
       </c>
-      <c r="B33" s="0" t="n">
+      <c r="B33" s="1" t="n">
         <v>32</v>
       </c>
-      <c r="C33" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D33" s="0" t="n">
+      <c r="C33" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" s="1" t="n">
         <v>2.5</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="n">
+      <c r="A34" s="1" t="n">
         <v>6406531910703</v>
       </c>
-      <c r="B34" s="0" t="n">
+      <c r="B34" s="1" t="n">
         <v>33</v>
       </c>
-      <c r="C34" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D34" s="0" t="n">
+      <c r="C34" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D34" s="1" t="n">
         <v>2.5</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="n">
+      <c r="A35" s="1" t="n">
         <v>6406531910704</v>
       </c>
-      <c r="B35" s="0" t="n">
+      <c r="B35" s="1" t="n">
         <v>34</v>
       </c>
-      <c r="C35" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D35" s="0" t="n">
+      <c r="C35" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D35" s="1" t="n">
         <v>2.5</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="n">
+      <c r="A36" s="1" t="n">
         <v>6406531910706</v>
       </c>
-      <c r="B36" s="0" t="n">
+      <c r="B36" s="1" t="n">
         <v>35</v>
       </c>
-      <c r="C36" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D36" s="0" t="n">
+      <c r="C36" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D36" s="1" t="n">
         <v>2.5</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="n">
+      <c r="A37" s="1" t="n">
         <v>6406531910707</v>
       </c>
-      <c r="B37" s="0" t="n">
+      <c r="B37" s="1" t="n">
         <v>36</v>
       </c>
-      <c r="C37" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D37" s="0" t="n">
+      <c r="C37" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D37" s="1" t="n">
         <v>2.5</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="n">
+      <c r="A38" s="1" t="n">
         <v>6406531910708</v>
       </c>
-      <c r="B38" s="0" t="n">
+      <c r="B38" s="1" t="n">
         <v>37</v>
       </c>
-      <c r="C38" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D38" s="0" t="n">
+      <c r="C38" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D38" s="1" t="n">
         <v>2.5</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="n">
+      <c r="A39" s="1" t="n">
         <v>6406531910710</v>
       </c>
-      <c r="B39" s="0" t="n">
+      <c r="B39" s="1" t="n">
         <v>38</v>
       </c>
-      <c r="C39" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D39" s="0" t="n">
+      <c r="C39" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D39" s="1" t="n">
         <v>2.5</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="n">
+      <c r="A40" s="1" t="n">
         <v>6406531910711</v>
       </c>
-      <c r="B40" s="0" t="n">
+      <c r="B40" s="1" t="n">
         <v>39</v>
       </c>
-      <c r="C40" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D40" s="0" t="n">
+      <c r="C40" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D40" s="1" t="n">
         <v>2.5</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="n">
+      <c r="A41" s="1" t="n">
         <v>6406531910712</v>
       </c>
-      <c r="B41" s="0" t="n">
+      <c r="B41" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="C41" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D41" s="0" t="n">
+      <c r="C41" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D41" s="1" t="n">
         <v>2.5</v>
       </c>
     </row>

</xml_diff>